<commit_message>
Employee test data updated
</commit_message>
<xml_diff>
--- a/data/employees.xlsx
+++ b/data/employees.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/335e73e05c013381/Desktop/AksSpace/BHR-QA-Automation/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shivam_PC\Desktop\Akshatha\BHR\BHR-QA-Automation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="11_E9C602311EC18124DCC317F030851802418E3E09" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43F3FFD4-8DB1-4960-9272-CBF0F36202F4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CF87A3-C453-418E-A90E-224E475EA8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25575" yWindow="17745" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>First name</t>
   </si>
@@ -55,58 +55,22 @@
     <t>2026-10-21</t>
   </si>
   <si>
-    <t>Tester</t>
-  </si>
-  <si>
-    <t>Emp2</t>
-  </si>
-  <si>
-    <t>Emp3</t>
-  </si>
-  <si>
-    <t>bhremp2@brighthr.com</t>
-  </si>
-  <si>
-    <t>bhremp3@brighthr.com</t>
-  </si>
-  <si>
-    <t>07564328974</t>
-  </si>
-  <si>
-    <t>07453876549</t>
-  </si>
-  <si>
-    <t>74534789765</t>
-  </si>
-  <si>
     <t>ProjectManager</t>
   </si>
   <si>
-    <t>SDET</t>
-  </si>
-  <si>
-    <t>JavaDeveloper</t>
-  </si>
-  <si>
-    <t>GW Developer</t>
-  </si>
-  <si>
-    <t>Emp4</t>
-  </si>
-  <si>
-    <t>Emp5</t>
-  </si>
-  <si>
-    <t>Emp6</t>
-  </si>
-  <si>
-    <t>bhremp4@brighthr.com</t>
-  </si>
-  <si>
-    <t>bhremp5@brighthr.com</t>
-  </si>
-  <si>
-    <t>bhremp6@brighthr.com</t>
+    <t>Emp7</t>
+  </si>
+  <si>
+    <t>Emp8</t>
+  </si>
+  <si>
+    <t>bhremp7@brighthr.com</t>
+  </si>
+  <si>
+    <t>bhremp8@brighthr.com</t>
+  </si>
+  <si>
+    <t>Senior SDET</t>
   </si>
 </sst>
 </file>
@@ -667,10 +631,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -991,15 +951,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="51.42578125" customWidth="1"/>
-    <col min="4" max="4" width="23.42578125" customWidth="1"/>
-    <col min="5" max="5" width="30.85546875" customWidth="1"/>
-    <col min="6" max="6" width="32.7109375" customWidth="1"/>
+    <col min="3" max="3" width="51.453125" customWidth="1"/>
+    <col min="4" max="4" width="23.453125" customWidth="1"/>
+    <col min="5" max="5" width="30.81640625" customWidth="1"/>
+    <col min="6" max="6" width="32.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1019,7 +979,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1036,10 +996,10 @@
         <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1056,70 +1016,22 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C4" s="1"/>
+      <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
-        <v>21</v>
-      </c>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C5" s="1"/>
+      <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="C6" s="1"/>
+      <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="E7" s="3"/>
     </row>
   </sheetData>
@@ -1127,9 +1039,6 @@
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{10E19B3C-73CB-43C8-B1C2-30B32E53CFDD}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{FC76E572-B949-488A-B8F0-4DA61C87C802}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{FB519803-65AA-4E20-9FC9-F6489B7E7107}"/>
-    <hyperlink ref="C6" r:id="rId4" xr:uid="{3905D8B6-DB15-4D8E-A25E-BD80350D8697}"/>
-    <hyperlink ref="C5" r:id="rId5" xr:uid="{F65C28BB-1239-49C7-9249-E39A924F70A3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>